<commit_message>
CV course exercises update
</commit_message>
<xml_diff>
--- a/training schedule.xlsx
+++ b/training schedule.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="78">
   <si>
     <t>Supervisor</t>
   </si>
@@ -233,25 +233,49 @@
     <t>6.5-12.5</t>
   </si>
   <si>
-    <t>13.5-</t>
+    <t>13.5-18.5</t>
+  </si>
+  <si>
+    <t>IMO the overlap with titanic is ok, if no visualization is required here</t>
+  </si>
+  <si>
+    <t>18.5-19.5</t>
+  </si>
+  <si>
+    <t>18.5-22.5</t>
+  </si>
+  <si>
+    <t>21.5-26.5</t>
+  </si>
+  <si>
+    <t>2.5?</t>
+  </si>
+  <si>
+    <t>27.5-29.5?</t>
+  </si>
+  <si>
+    <t>28.5-4.6?</t>
+  </si>
+  <si>
+    <t>29-4.6?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="177"/>
       <scheme val="minor"/>
@@ -259,7 +283,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -267,7 +291,7 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -275,14 +299,21 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -318,7 +349,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -415,6 +446,15 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -424,7 +464,7 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -487,6 +527,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="20% - הדגשה1" xfId="3" builtinId="30"/>
@@ -496,7 +548,54 @@
     <cellStyle name="Normal 2" xfId="1"/>
     <cellStyle name="הדגשה1" xfId="2" builtinId="29"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="25">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF33CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <gradientFill>
+          <stop position="0">
+            <color rgb="FFFF66CC"/>
+          </stop>
+          <stop position="1">
+            <color theme="5" tint="0.40000610370189521"/>
+          </stop>
+        </gradientFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -969,20 +1068,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I64"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.9140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.25" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.26953125" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.9140625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="17.33203125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="12.25" style="2" customWidth="1"/>
-    <col min="9" max="9" width="25.4140625" customWidth="1"/>
+    <col min="4" max="4" width="14.36328125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.90625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="17.36328125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="13.36328125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="12.26953125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="25.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="22" t="s">
         <v>27</v>
       </c>
@@ -1011,7 +1110,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="17" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" s="17" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
         <v>3</v>
       </c>
@@ -1021,7 +1120,7 @@
       </c>
       <c r="C2" s="20">
         <f>SUM(C3:C8)</f>
-        <v>6.5</v>
+        <v>10</v>
       </c>
       <c r="D2" s="20"/>
       <c r="E2" s="20"/>
@@ -1030,7 +1129,7 @@
       <c r="H2" s="20"/>
       <c r="I2" s="20"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>33</v>
       </c>
@@ -1057,7 +1156,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
@@ -1082,7 +1181,7 @@
       </c>
       <c r="I4" s="24"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
@@ -1109,7 +1208,7 @@
       </c>
       <c r="I5" s="24"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
@@ -1135,7 +1234,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
@@ -1164,28 +1263,42 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="8">
         <v>5</v>
       </c>
-      <c r="C8" s="8"/>
+      <c r="C8" s="8">
+        <v>3.5</v>
+      </c>
       <c r="D8" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="F8" s="2">
+        <v>2</v>
+      </c>
+      <c r="G8" s="2">
+        <v>4</v>
+      </c>
+      <c r="H8" s="2">
+        <v>4</v>
+      </c>
+      <c r="I8" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="9"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
       <c r="D9" s="21"/>
     </row>
-    <row r="10" spans="1:9" s="17" customFormat="1" ht="28.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" s="17" customFormat="1" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="18" t="s">
         <v>34</v>
       </c>
@@ -1198,13 +1311,15 @@
         <v>0</v>
       </c>
       <c r="D10" s="16"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="29"/>
-      <c r="I10"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E10" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" s="33"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="33"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>42</v>
       </c>
@@ -1215,9 +1330,13 @@
       <c r="D11" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F11" s="1"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E11" s="32"/>
+      <c r="F11" s="33"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="33"/>
+      <c r="I11" s="33"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>41</v>
       </c>
@@ -1228,8 +1347,13 @@
       <c r="D12" s="4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E12" s="32"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="33"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>40</v>
       </c>
@@ -1240,8 +1364,13 @@
       <c r="D13" s="4" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E13" s="32"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="33"/>
+      <c r="H13" s="33"/>
+      <c r="I13" s="33"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>39</v>
       </c>
@@ -1252,8 +1381,13 @@
       <c r="D14" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E14" s="32"/>
+      <c r="F14" s="33"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="33"/>
+      <c r="I14" s="33"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>38</v>
       </c>
@@ -1264,8 +1398,13 @@
       <c r="D15" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E15" s="32"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="33"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>37</v>
       </c>
@@ -1276,8 +1415,13 @@
       <c r="D16" s="4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E16" s="32"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>36</v>
       </c>
@@ -1288,8 +1432,13 @@
       <c r="D17" s="4" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E17" s="32"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="33"/>
+      <c r="I17" s="33"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
         <v>35</v>
       </c>
@@ -1300,14 +1449,19 @@
       <c r="D18" s="8" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E18" s="32"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="33"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" s="9"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
       <c r="D19" s="21"/>
     </row>
-    <row r="20" spans="1:8" s="17" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" s="17" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="15" t="s">
         <v>28</v>
       </c>
@@ -1317,7 +1471,7 @@
       </c>
       <c r="C20" s="16">
         <f>SUM(C21,C29,C30)</f>
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="D20" s="16"/>
       <c r="E20" s="2"/>
@@ -1325,7 +1479,7 @@
       <c r="G20" s="29"/>
       <c r="H20" s="29"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
         <v>30</v>
       </c>
@@ -1335,60 +1489,116 @@
       </c>
       <c r="C21" s="6">
         <f>SUM(C22:C28)</f>
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="D21" s="6"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>45</v>
       </c>
       <c r="B22" s="4">
         <v>1</v>
       </c>
-      <c r="C22" s="4"/>
+      <c r="C22" s="4">
+        <v>0.5</v>
+      </c>
       <c r="D22" s="4" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E22" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F22" s="2">
+        <v>4</v>
+      </c>
+      <c r="G22" s="2">
+        <v>4</v>
+      </c>
+      <c r="H22" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>46</v>
       </c>
       <c r="B23" s="4">
         <v>2.5</v>
       </c>
-      <c r="C23" s="4"/>
+      <c r="C23" s="4">
+        <v>3</v>
+      </c>
       <c r="D23" s="4" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E23" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F23" s="2">
+        <v>3</v>
+      </c>
+      <c r="G23" s="2">
+        <v>4</v>
+      </c>
+      <c r="H23" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>47</v>
       </c>
       <c r="B24" s="4">
         <v>2.5</v>
       </c>
-      <c r="C24" s="4"/>
+      <c r="C24" s="4">
+        <v>3</v>
+      </c>
       <c r="D24" s="4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E24" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F24" s="2">
+        <v>4</v>
+      </c>
+      <c r="G24" s="2">
+        <v>5</v>
+      </c>
+      <c r="H24" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>48</v>
       </c>
       <c r="B25" s="4">
         <v>4</v>
       </c>
-      <c r="C25" s="4"/>
+      <c r="C25" s="31" t="s">
+        <v>74</v>
+      </c>
       <c r="D25" s="4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
+      <c r="E25" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F25" s="2">
+        <v>4</v>
+      </c>
+      <c r="G25" s="2">
+        <v>4</v>
+      </c>
+      <c r="H25" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" s="30" t="s">
         <v>49</v>
       </c>
       <c r="B26" s="4">
@@ -1398,8 +1608,20 @@
       <c r="D26" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E26" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F26" s="2">
+        <v>2</v>
+      </c>
+      <c r="G26" s="2">
+        <v>4</v>
+      </c>
+      <c r="H26" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>50</v>
       </c>
@@ -1410,8 +1632,20 @@
       <c r="D27" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E27" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F27" s="2">
+        <v>1</v>
+      </c>
+      <c r="G27" s="2">
+        <v>5</v>
+      </c>
+      <c r="H27" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
         <v>51</v>
       </c>
@@ -1423,7 +1657,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
         <v>43</v>
       </c>
@@ -1435,7 +1669,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" s="13" t="s">
         <v>44</v>
       </c>
@@ -1447,13 +1681,13 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" s="9"/>
       <c r="B31" s="10"/>
       <c r="C31" s="10"/>
       <c r="D31" s="21"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" s="15" t="s">
         <v>29</v>
       </c>
@@ -1467,7 +1701,7 @@
       </c>
       <c r="D32" s="16"/>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
         <v>30</v>
       </c>
@@ -1481,7 +1715,7 @@
       </c>
       <c r="D33" s="6"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
         <v>12</v>
       </c>
@@ -1493,7 +1727,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
         <v>13</v>
       </c>
@@ -1505,7 +1739,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
         <v>14</v>
       </c>
@@ -1517,7 +1751,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>15</v>
       </c>
@@ -1529,7 +1763,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
         <v>16</v>
       </c>
@@ -1541,7 +1775,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>17</v>
       </c>
@@ -1553,7 +1787,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
         <v>31</v>
       </c>
@@ -1566,7 +1800,7 @@
       </c>
       <c r="D40" s="6"/>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
         <v>18</v>
       </c>
@@ -1576,7 +1810,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
         <v>19</v>
       </c>
@@ -1586,7 +1820,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
@@ -1596,7 +1830,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" s="13" t="s">
         <v>32</v>
       </c>
@@ -1606,13 +1840,13 @@
       <c r="C44" s="14"/>
       <c r="D44" s="14"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" s="9"/>
       <c r="B45" s="10"/>
       <c r="C45" s="10"/>
       <c r="D45" s="21"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" s="15" t="s">
         <v>1</v>
       </c>
@@ -1620,10 +1854,13 @@
         <f>SUM(B47)</f>
         <v>0.5</v>
       </c>
-      <c r="C46" s="16"/>
+      <c r="C46" s="16">
+        <f>SUM(C47:C49)</f>
+        <v>1</v>
+      </c>
       <c r="D46" s="16"/>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" s="11" t="s">
         <v>2</v>
       </c>
@@ -1643,11 +1880,14 @@
       <c r="G47" s="2">
         <v>4</v>
       </c>
+      <c r="H47" s="2">
+        <v>4</v>
+      </c>
       <c r="I47" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" s="25" t="s">
         <v>52</v>
       </c>
@@ -1664,8 +1904,14 @@
       <c r="F48" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G48" s="2">
+        <v>3</v>
+      </c>
+      <c r="H48" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" s="25" t="s">
         <v>54</v>
       </c>
@@ -1692,49 +1938,72 @@
         <v>55</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="C55" s="1"/>
       <c r="D55" s="1"/>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="C56" s="1"/>
       <c r="D56" s="1"/>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="C57" s="1"/>
       <c r="D57" s="1"/>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
       <c r="C64" s="1"/>
       <c r="D64" s="1"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E10:I18"/>
+  </mergeCells>
   <conditionalFormatting sqref="D41">
-    <cfRule type="cellIs" dxfId="18" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="20" operator="equal">
       <formula>"Hadar and Yaniv"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1:D47 D50:D1048576 E1:I2">
+  <conditionalFormatting sqref="D1:D23 D50:D1048576 E1:I2 D27:D47">
+    <cfRule type="cellIs" dxfId="23" priority="19" operator="equal">
+      <formula>"yoni and david"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="21" operator="equal">
+      <formula>"yoni"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="22" operator="equal">
+      <formula>"hadar"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="20" priority="23" operator="equal">
+      <formula>"david"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="19" priority="24" operator="equal">
+      <formula>"itay"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="18" priority="25" operator="equal">
+      <formula>"yaniv"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D48">
     <cfRule type="cellIs" dxfId="17" priority="13" operator="equal">
       <formula>"yoni and david"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="14" operator="equal">
       <formula>"yoni"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="15" operator="equal">
       <formula>"hadar"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="16" operator="equal">
       <formula>"david"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="17" operator="equal">
       <formula>"itay"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="18" operator="equal">
       <formula>"yaniv"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D48">
+  <conditionalFormatting sqref="D49">
     <cfRule type="cellIs" dxfId="11" priority="7" operator="equal">
       <formula>"yoni and david"</formula>
     </cfRule>
@@ -1754,7 +2023,7 @@
       <formula>"yaniv"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D49">
+  <conditionalFormatting sqref="D24:D26">
     <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <formula>"yoni and david"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Finished deep, starting RCNN papers
</commit_message>
<xml_diff>
--- a/training schedule.xlsx
+++ b/training schedule.xlsx
@@ -1,30 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\CV Training Guy\CV_training\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guyle\Documents\Projects\CV_training\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA4FB744-BC6D-4AC3-8D5C-C4542E55060C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14380" windowHeight="4220"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="84">
   <si>
     <t>Supervisor</t>
   </si>
@@ -269,16 +281,19 @@
     <t>some minor compatibility issues, I think second notebook (two stage detector) is redundant after first notebook (one stage detector)</t>
   </si>
   <si>
-    <t>1.7-?</t>
-  </si>
-  <si>
-    <t>26.6-1.7?</t>
+    <t>1.7-6.7</t>
+  </si>
+  <si>
+    <t>26.6-1.7</t>
+  </si>
+  <si>
+    <t>6.7-</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -560,14 +575,61 @@
     </xf>
   </cellXfs>
   <cellStyles count="6">
-    <cellStyle name="20% - הדגשה1" xfId="3" builtinId="30"/>
-    <cellStyle name="40% - הדגשה1" xfId="4" builtinId="31"/>
-    <cellStyle name="60% - הדגשה1" xfId="5" builtinId="32"/>
+    <cellStyle name="20% - Accent1" xfId="3" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="4" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="5" builtinId="32"/>
+    <cellStyle name="Accent1" xfId="2" builtinId="29"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
-    <cellStyle name="הדגשה1" xfId="2" builtinId="29"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
   </cellStyles>
-  <dxfs count="32">
+  <dxfs count="13">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF33CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <gradientFill>
+          <stop position="0">
+            <color rgb="FFFF66CC"/>
+          </stop>
+          <stop position="1">
+            <color theme="5" tint="0.40000610370189521"/>
+          </stop>
+        </gradientFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <gradientFill>
@@ -623,206 +685,6 @@
           </stop>
           <stop position="1">
             <color theme="5" tint="0.40000610370189521"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF33CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill>
-          <stop position="0">
-            <color rgb="FFFF66CC"/>
-          </stop>
-          <stop position="1">
-            <color theme="5" tint="0.40000610370189521"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF33CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill>
-          <stop position="0">
-            <color rgb="FFFF66CC"/>
-          </stop>
-          <stop position="1">
-            <color theme="5" tint="0.40000610370189521"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF33CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill>
-          <stop position="0">
-            <color rgb="FFFF66CC"/>
-          </stop>
-          <stop position="1">
-            <color theme="5" tint="0.40000610370189521"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF33CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill>
-          <stop position="0">
-            <color rgb="FFFF66CC"/>
-          </stop>
-          <stop position="1">
-            <color theme="5" tint="0.40000610370189521"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill>
-          <stop position="0">
-            <color rgb="FF33CCCC"/>
-          </stop>
-          <stop position="1">
-            <color theme="9" tint="0.40000610370189521"/>
           </stop>
         </gradientFill>
       </fill>
@@ -1144,17 +1006,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I64"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.26953125" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.36328125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.453125" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.1796875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="17.36328125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="17.453125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="13.453125" style="2" customWidth="1"/>
     <col min="8" max="8" width="12.26953125" style="2" customWidth="1"/>
     <col min="9" max="9" width="25.453125" customWidth="1"/>
   </cols>
@@ -1807,7 +1669,7 @@
       </c>
       <c r="C32" s="16">
         <f>SUM(C33,C40,C44)</f>
-        <v>9.5</v>
+        <v>15</v>
       </c>
       <c r="D32" s="16"/>
     </row>
@@ -1821,7 +1683,7 @@
       </c>
       <c r="C33" s="6">
         <f>SUM(C34:C39)</f>
-        <v>9.5</v>
+        <v>15</v>
       </c>
       <c r="D33" s="6"/>
     </row>
@@ -1925,12 +1787,23 @@
       <c r="B38" s="4">
         <v>3.5</v>
       </c>
-      <c r="C38" s="4"/>
+      <c r="C38" s="4">
+        <v>3.5</v>
+      </c>
       <c r="D38" s="4" t="s">
         <v>11</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>82</v>
+      </c>
+      <c r="F38" s="2">
+        <v>4</v>
+      </c>
+      <c r="G38" s="2">
+        <v>5</v>
+      </c>
+      <c r="H38" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.35">
@@ -1940,12 +1813,23 @@
       <c r="B39" s="4">
         <v>2.5</v>
       </c>
-      <c r="C39" s="4"/>
+      <c r="C39" s="4">
+        <v>2</v>
+      </c>
       <c r="D39" s="4" t="s">
         <v>6</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>81</v>
+      </c>
+      <c r="F39" s="2">
+        <v>4</v>
+      </c>
+      <c r="G39" s="2">
+        <v>5</v>
+      </c>
+      <c r="H39" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.35">
@@ -1969,6 +1853,9 @@
       <c r="C41" s="4"/>
       <c r="D41" s="4" t="s">
         <v>23</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
@@ -2119,109 +2006,49 @@
   <mergeCells count="1">
     <mergeCell ref="E10:I18"/>
   </mergeCells>
-  <conditionalFormatting sqref="D1:D23 D50:D1048576 E1:I2 D27:D31 D45:D47">
-    <cfRule type="cellIs" dxfId="30" priority="26" operator="equal">
+  <conditionalFormatting sqref="D1:D1048576">
+    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
       <formula>"yoni and david"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="29" priority="28" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="2" operator="equal">
       <formula>"yoni"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="29" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="3" operator="equal">
       <formula>"hadar"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="4" operator="equal">
       <formula>"david"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="31" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="5" operator="equal">
       <formula>"itay"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="32" operator="equal">
-      <formula>"yaniv"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D48">
-    <cfRule type="cellIs" dxfId="24" priority="20" operator="equal">
-      <formula>"yoni and david"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="23" priority="21" operator="equal">
-      <formula>"yoni"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="22" operator="equal">
-      <formula>"hadar"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="23" operator="equal">
-      <formula>"david"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="24" operator="equal">
-      <formula>"itay"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="25" operator="equal">
-      <formula>"yaniv"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D49">
-    <cfRule type="cellIs" dxfId="18" priority="14" operator="equal">
-      <formula>"yoni and david"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="15" operator="equal">
-      <formula>"yoni"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="16" operator="equal">
-      <formula>"hadar"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="17" operator="equal">
-      <formula>"david"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="18" operator="equal">
-      <formula>"itay"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="19" operator="equal">
-      <formula>"yaniv"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D24:D26">
-    <cfRule type="cellIs" dxfId="12" priority="8" operator="equal">
-      <formula>"yoni and david"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="9" operator="equal">
-      <formula>"yoni"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="10" operator="equal">
-      <formula>"hadar"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="11" operator="equal">
-      <formula>"david"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="12" operator="equal">
-      <formula>"itay"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="13" operator="equal">
-      <formula>"yaniv"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D32:D44">
-    <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
-      <formula>"yoni and david"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
-      <formula>"yoni"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
-      <formula>"hadar"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
-      <formula>"david"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="5" operator="equal">
-      <formula>"itay"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="6" operator="equal">
       <formula>"yaniv"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D41">
-    <cfRule type="cellIs" dxfId="0" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
       <formula>"Hadar and Yaniv"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E1:I2">
+    <cfRule type="cellIs" dxfId="5" priority="26" operator="equal">
+      <formula>"yoni and david"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="28" operator="equal">
+      <formula>"yoni"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="29" operator="equal">
+      <formula>"hadar"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="30" operator="equal">
+      <formula>"david"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="31" operator="equal">
+      <formula>"itay"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="32" operator="equal">
+      <formula>"yaniv"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>